<commit_message>
Update Code For Dashboard Admin
</commit_message>
<xml_diff>
--- a/outputs/01a0798e-2dd6-7ab0-8fa5-cb4fd27e035e/product-import-template.xlsx
+++ b/outputs/01a0798e-2dd6-7ab0-8fa5-cb4fd27e035e/product-import-template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="1" r:id="R3b49490a5cdd4271"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="2" r:id="R50f660f0d6f849cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="3" r:id="Ree684f17850c47d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specifications" sheetId="4" r:id="Rcfdfff0810b84371"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="5" r:id="R09fb66156daf422e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="1" r:id="Rf0d6a90fb4c04da2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="2" r:id="Re84482ac938e413d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="3" r:id="R6b680bf8e20c4b46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specifications" sheetId="4" r:id="R7bda9e173e7d4805"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="5" r:id="Rd1e538c1331c428f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -430,14 +430,15 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="VariantsTable" displayName="VariantsTable" ref="A4:F23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="6">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="VariantsTable" displayName="VariantsTable" ref="A4:G23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
     <x:tableColumn id="1" name="product_sku"/>
     <x:tableColumn id="2" name="variant_sku"/>
     <x:tableColumn id="3" name="attribute_values"/>
     <x:tableColumn id="4" name="price"/>
     <x:tableColumn id="5" name="sale_price"/>
-    <x:tableColumn id="6" name="is_active"/>
+    <x:tableColumn id="6" name="stock"/>
+    <x:tableColumn id="7" name="is_active"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -738,7 +739,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="54" t="str">
-        <x:v>Sản phẩm variant phải có ít nhất một dòng ở Variants; attribute_values dùng Attribute=Value;Attribute=Value.</x:v>
+        <x:v>Sản phẩm variant phải có ít nhất một dòng ở Variants; stock của từng dòng đặt trong Variants; attribute_values dùng Attribute=Value;Attribute=Value.</x:v>
       </x:c>
       <x:c r="C8" s="54" t="str"/>
       <x:c r="D8" s="54" t="str"/>
@@ -832,7 +833,7 @@
         <x:v>Variants</x:v>
       </x:c>
       <x:c r="B15" s="27" t="str">
-        <x:v>Variant prices and attributes</x:v>
+        <x:v>Variant prices, stock and attributes</x:v>
       </x:c>
       <x:c r="C15" s="27" t="str">
         <x:v>All headers in row 4</x:v>
@@ -1057,9 +1058,7 @@
       <x:c r="E5" s="33" t="str">
         <x:v>variant</x:v>
       </x:c>
-      <x:c r="F5" s="41" t="n">
-        <x:v>18</x:v>
-      </x:c>
+      <x:c r="F5" s="41" t="str"/>
       <x:c r="G5" s="41" t="str"/>
       <x:c r="H5" s="41" t="str"/>
       <x:c r="I5" s="33" t="str"/>
@@ -1996,7 +1995,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91413a0956bb4668"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R611f3f1ccb2446f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2011,6 +2010,7 @@
     <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -2021,17 +2021,19 @@
       <x:c r="C1" s="62"/>
       <x:c r="D1" s="62"/>
       <x:c r="E1" s="62"/>
-      <x:c r="F1" s="63"/>
+      <x:c r="F1" s="62"/>
+      <x:c r="G1" s="63"/>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="64" t="str">
-        <x:v>Chỉ dùng cho sản phẩm type=variant. Mỗi dòng là một tổ hợp thuộc tính duy nhất.</x:v>
+        <x:v>Chỉ dùng cho sản phẩm type=variant. Mỗi dòng là một tổ hợp thuộc tính duy nhất; stock là tồn kho riêng của từng biến thể.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
       <x:c r="D2" s="7"/>
       <x:c r="E2" s="7"/>
-      <x:c r="F2" s="65"/>
+      <x:c r="F2" s="7"/>
+      <x:c r="G2" s="65"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="66"/>
@@ -2039,7 +2041,8 @@
       <x:c r="C3" s="67"/>
       <x:c r="D3" s="67"/>
       <x:c r="E3" s="67"/>
-      <x:c r="F3" s="68"/>
+      <x:c r="F3" s="67"/>
+      <x:c r="G3" s="68"/>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -2058,6 +2061,9 @@
         <x:v>sale_price</x:v>
       </x:c>
       <x:c r="F4" s="12" t="str">
+        <x:v>stock</x:v>
+      </x:c>
+      <x:c r="G4" s="12" t="str">
         <x:v>is_active</x:v>
       </x:c>
     </x:row>
@@ -2076,6 +2082,9 @@
       </x:c>
       <x:c r="E5" s="41" t="str"/>
       <x:c r="F5" s="33" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G5" s="33" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -2096,6 +2105,9 @@
         <x:v>35990000</x:v>
       </x:c>
       <x:c r="F6" s="36" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G6" s="36" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -2106,6 +2118,7 @@
       <x:c r="D7" s="42" t="str"/>
       <x:c r="E7" s="42" t="str"/>
       <x:c r="F7" s="36" t="str"/>
+      <x:c r="G7" s="36" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="36" t="str"/>
@@ -2114,6 +2127,7 @@
       <x:c r="D8" s="42" t="str"/>
       <x:c r="E8" s="42" t="str"/>
       <x:c r="F8" s="36" t="str"/>
+      <x:c r="G8" s="36" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="36" t="str"/>
@@ -2122,6 +2136,7 @@
       <x:c r="D9" s="42" t="str"/>
       <x:c r="E9" s="42" t="str"/>
       <x:c r="F9" s="36" t="str"/>
+      <x:c r="G9" s="36" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="36" t="str"/>
@@ -2130,6 +2145,7 @@
       <x:c r="D10" s="42" t="str"/>
       <x:c r="E10" s="42" t="str"/>
       <x:c r="F10" s="36" t="str"/>
+      <x:c r="G10" s="36" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="36" t="str"/>
@@ -2138,6 +2154,7 @@
       <x:c r="D11" s="42" t="str"/>
       <x:c r="E11" s="42" t="str"/>
       <x:c r="F11" s="36" t="str"/>
+      <x:c r="G11" s="36" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="36" t="str"/>
@@ -2146,6 +2163,7 @@
       <x:c r="D12" s="42" t="str"/>
       <x:c r="E12" s="42" t="str"/>
       <x:c r="F12" s="36" t="str"/>
+      <x:c r="G12" s="36" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="36" t="str"/>
@@ -2154,6 +2172,7 @@
       <x:c r="D13" s="42" t="str"/>
       <x:c r="E13" s="42" t="str"/>
       <x:c r="F13" s="36" t="str"/>
+      <x:c r="G13" s="36" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="36" t="str"/>
@@ -2162,6 +2181,7 @@
       <x:c r="D14" s="42" t="str"/>
       <x:c r="E14" s="42" t="str"/>
       <x:c r="F14" s="36" t="str"/>
+      <x:c r="G14" s="36" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="36" t="str"/>
@@ -2170,6 +2190,7 @@
       <x:c r="D15" s="42" t="str"/>
       <x:c r="E15" s="42" t="str"/>
       <x:c r="F15" s="36" t="str"/>
+      <x:c r="G15" s="36" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="36" t="str"/>
@@ -2178,6 +2199,7 @@
       <x:c r="D16" s="42" t="str"/>
       <x:c r="E16" s="42" t="str"/>
       <x:c r="F16" s="36" t="str"/>
+      <x:c r="G16" s="36" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="36" t="str"/>
@@ -2186,6 +2208,7 @@
       <x:c r="D17" s="42" t="str"/>
       <x:c r="E17" s="42" t="str"/>
       <x:c r="F17" s="36" t="str"/>
+      <x:c r="G17" s="36" t="str"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="36" t="str"/>
@@ -2194,6 +2217,7 @@
       <x:c r="D18" s="42" t="str"/>
       <x:c r="E18" s="42" t="str"/>
       <x:c r="F18" s="36" t="str"/>
+      <x:c r="G18" s="36" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="36" t="str"/>
@@ -2202,6 +2226,7 @@
       <x:c r="D19" s="42" t="str"/>
       <x:c r="E19" s="42" t="str"/>
       <x:c r="F19" s="36" t="str"/>
+      <x:c r="G19" s="36" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="36" t="str"/>
@@ -2210,6 +2235,7 @@
       <x:c r="D20" s="42" t="str"/>
       <x:c r="E20" s="42" t="str"/>
       <x:c r="F20" s="36" t="str"/>
+      <x:c r="G20" s="36" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="36" t="str"/>
@@ -2218,6 +2244,7 @@
       <x:c r="D21" s="42" t="str"/>
       <x:c r="E21" s="42" t="str"/>
       <x:c r="F21" s="36" t="str"/>
+      <x:c r="G21" s="36" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="36" t="str"/>
@@ -2226,6 +2253,7 @@
       <x:c r="D22" s="42" t="str"/>
       <x:c r="E22" s="42" t="str"/>
       <x:c r="F22" s="36" t="str"/>
+      <x:c r="G22" s="36" t="str"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="39" t="str"/>
@@ -2234,6 +2262,7 @@
       <x:c r="D23" s="43" t="str"/>
       <x:c r="E23" s="43" t="str"/>
       <x:c r="F23" s="39" t="str"/>
+      <x:c r="G23" s="39" t="str"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="66"/>
@@ -2241,7 +2270,8 @@
       <x:c r="C24" s="67"/>
       <x:c r="D24" s="44"/>
       <x:c r="E24" s="44"/>
-      <x:c r="F24" s="68"/>
+      <x:c r="F24" s="67"/>
+      <x:c r="G24" s="68"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="66"/>
@@ -2249,7 +2279,8 @@
       <x:c r="C25" s="67"/>
       <x:c r="D25" s="44"/>
       <x:c r="E25" s="44"/>
-      <x:c r="F25" s="68"/>
+      <x:c r="F25" s="67"/>
+      <x:c r="G25" s="68"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="66"/>
@@ -2257,7 +2288,8 @@
       <x:c r="C26" s="67"/>
       <x:c r="D26" s="44"/>
       <x:c r="E26" s="44"/>
-      <x:c r="F26" s="68"/>
+      <x:c r="F26" s="67"/>
+      <x:c r="G26" s="68"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="66"/>
@@ -2265,7 +2297,8 @@
       <x:c r="C27" s="67"/>
       <x:c r="D27" s="44"/>
       <x:c r="E27" s="44"/>
-      <x:c r="F27" s="68"/>
+      <x:c r="F27" s="67"/>
+      <x:c r="G27" s="68"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="66"/>
@@ -2273,7 +2306,8 @@
       <x:c r="C28" s="67"/>
       <x:c r="D28" s="44"/>
       <x:c r="E28" s="44"/>
-      <x:c r="F28" s="68"/>
+      <x:c r="F28" s="67"/>
+      <x:c r="G28" s="68"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="66"/>
@@ -2281,7 +2315,8 @@
       <x:c r="C29" s="67"/>
       <x:c r="D29" s="44"/>
       <x:c r="E29" s="44"/>
-      <x:c r="F29" s="68"/>
+      <x:c r="F29" s="67"/>
+      <x:c r="G29" s="68"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="66"/>
@@ -2289,7 +2324,8 @@
       <x:c r="C30" s="67"/>
       <x:c r="D30" s="44"/>
       <x:c r="E30" s="44"/>
-      <x:c r="F30" s="68"/>
+      <x:c r="F30" s="67"/>
+      <x:c r="G30" s="68"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="66"/>
@@ -2297,7 +2333,8 @@
       <x:c r="C31" s="67"/>
       <x:c r="D31" s="44"/>
       <x:c r="E31" s="44"/>
-      <x:c r="F31" s="68"/>
+      <x:c r="F31" s="67"/>
+      <x:c r="G31" s="68"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="66"/>
@@ -2305,7 +2342,8 @@
       <x:c r="C32" s="67"/>
       <x:c r="D32" s="44"/>
       <x:c r="E32" s="44"/>
-      <x:c r="F32" s="68"/>
+      <x:c r="F32" s="67"/>
+      <x:c r="G32" s="68"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="66"/>
@@ -2313,7 +2351,8 @@
       <x:c r="C33" s="67"/>
       <x:c r="D33" s="44"/>
       <x:c r="E33" s="44"/>
-      <x:c r="F33" s="68"/>
+      <x:c r="F33" s="67"/>
+      <x:c r="G33" s="68"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="66"/>
@@ -2321,7 +2360,8 @@
       <x:c r="C34" s="67"/>
       <x:c r="D34" s="44"/>
       <x:c r="E34" s="44"/>
-      <x:c r="F34" s="68"/>
+      <x:c r="F34" s="67"/>
+      <x:c r="G34" s="68"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="66"/>
@@ -2329,7 +2369,8 @@
       <x:c r="C35" s="67"/>
       <x:c r="D35" s="44"/>
       <x:c r="E35" s="44"/>
-      <x:c r="F35" s="68"/>
+      <x:c r="F35" s="67"/>
+      <x:c r="G35" s="68"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="66"/>
@@ -2337,7 +2378,8 @@
       <x:c r="C36" s="67"/>
       <x:c r="D36" s="44"/>
       <x:c r="E36" s="44"/>
-      <x:c r="F36" s="68"/>
+      <x:c r="F36" s="67"/>
+      <x:c r="G36" s="68"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="66"/>
@@ -2345,7 +2387,8 @@
       <x:c r="C37" s="67"/>
       <x:c r="D37" s="44"/>
       <x:c r="E37" s="44"/>
-      <x:c r="F37" s="68"/>
+      <x:c r="F37" s="67"/>
+      <x:c r="G37" s="68"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="66"/>
@@ -2353,7 +2396,8 @@
       <x:c r="C38" s="67"/>
       <x:c r="D38" s="44"/>
       <x:c r="E38" s="44"/>
-      <x:c r="F38" s="68"/>
+      <x:c r="F38" s="67"/>
+      <x:c r="G38" s="68"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="66"/>
@@ -2361,7 +2405,8 @@
       <x:c r="C39" s="67"/>
       <x:c r="D39" s="44"/>
       <x:c r="E39" s="44"/>
-      <x:c r="F39" s="68"/>
+      <x:c r="F39" s="67"/>
+      <x:c r="G39" s="68"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="66"/>
@@ -2369,7 +2414,8 @@
       <x:c r="C40" s="67"/>
       <x:c r="D40" s="44"/>
       <x:c r="E40" s="44"/>
-      <x:c r="F40" s="68"/>
+      <x:c r="F40" s="67"/>
+      <x:c r="G40" s="68"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="66"/>
@@ -2377,7 +2423,8 @@
       <x:c r="C41" s="67"/>
       <x:c r="D41" s="44"/>
       <x:c r="E41" s="44"/>
-      <x:c r="F41" s="68"/>
+      <x:c r="F41" s="67"/>
+      <x:c r="G41" s="68"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="66"/>
@@ -2385,7 +2432,8 @@
       <x:c r="C42" s="67"/>
       <x:c r="D42" s="44"/>
       <x:c r="E42" s="44"/>
-      <x:c r="F42" s="68"/>
+      <x:c r="F42" s="67"/>
+      <x:c r="G42" s="68"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="66"/>
@@ -2393,7 +2441,8 @@
       <x:c r="C43" s="67"/>
       <x:c r="D43" s="44"/>
       <x:c r="E43" s="44"/>
-      <x:c r="F43" s="68"/>
+      <x:c r="F43" s="67"/>
+      <x:c r="G43" s="68"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="66"/>
@@ -2401,7 +2450,8 @@
       <x:c r="C44" s="67"/>
       <x:c r="D44" s="44"/>
       <x:c r="E44" s="44"/>
-      <x:c r="F44" s="68"/>
+      <x:c r="F44" s="67"/>
+      <x:c r="G44" s="68"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="66"/>
@@ -2409,7 +2459,8 @@
       <x:c r="C45" s="67"/>
       <x:c r="D45" s="44"/>
       <x:c r="E45" s="44"/>
-      <x:c r="F45" s="68"/>
+      <x:c r="F45" s="67"/>
+      <x:c r="G45" s="68"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="66"/>
@@ -2417,7 +2468,8 @@
       <x:c r="C46" s="67"/>
       <x:c r="D46" s="44"/>
       <x:c r="E46" s="44"/>
-      <x:c r="F46" s="68"/>
+      <x:c r="F46" s="67"/>
+      <x:c r="G46" s="68"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="66"/>
@@ -2425,7 +2477,8 @@
       <x:c r="C47" s="67"/>
       <x:c r="D47" s="44"/>
       <x:c r="E47" s="44"/>
-      <x:c r="F47" s="68"/>
+      <x:c r="F47" s="67"/>
+      <x:c r="G47" s="68"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="66"/>
@@ -2433,7 +2486,8 @@
       <x:c r="C48" s="67"/>
       <x:c r="D48" s="44"/>
       <x:c r="E48" s="44"/>
-      <x:c r="F48" s="68"/>
+      <x:c r="F48" s="67"/>
+      <x:c r="G48" s="68"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="66"/>
@@ -2441,7 +2495,8 @@
       <x:c r="C49" s="67"/>
       <x:c r="D49" s="44"/>
       <x:c r="E49" s="44"/>
-      <x:c r="F49" s="68"/>
+      <x:c r="F49" s="67"/>
+      <x:c r="G49" s="68"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="66"/>
@@ -2449,7 +2504,8 @@
       <x:c r="C50" s="67"/>
       <x:c r="D50" s="44"/>
       <x:c r="E50" s="44"/>
-      <x:c r="F50" s="68"/>
+      <x:c r="F50" s="67"/>
+      <x:c r="G50" s="68"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="66"/>
@@ -2457,7 +2513,8 @@
       <x:c r="C51" s="67"/>
       <x:c r="D51" s="44"/>
       <x:c r="E51" s="44"/>
-      <x:c r="F51" s="68"/>
+      <x:c r="F51" s="67"/>
+      <x:c r="G51" s="68"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="66"/>
@@ -2465,7 +2522,8 @@
       <x:c r="C52" s="67"/>
       <x:c r="D52" s="44"/>
       <x:c r="E52" s="44"/>
-      <x:c r="F52" s="68"/>
+      <x:c r="F52" s="67"/>
+      <x:c r="G52" s="68"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="66"/>
@@ -2473,7 +2531,8 @@
       <x:c r="C53" s="67"/>
       <x:c r="D53" s="44"/>
       <x:c r="E53" s="44"/>
-      <x:c r="F53" s="68"/>
+      <x:c r="F53" s="67"/>
+      <x:c r="G53" s="68"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="66"/>
@@ -2481,7 +2540,8 @@
       <x:c r="C54" s="67"/>
       <x:c r="D54" s="44"/>
       <x:c r="E54" s="44"/>
-      <x:c r="F54" s="68"/>
+      <x:c r="F54" s="67"/>
+      <x:c r="G54" s="68"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="66"/>
@@ -2489,7 +2549,8 @@
       <x:c r="C55" s="67"/>
       <x:c r="D55" s="44"/>
       <x:c r="E55" s="44"/>
-      <x:c r="F55" s="68"/>
+      <x:c r="F55" s="67"/>
+      <x:c r="G55" s="68"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="66"/>
@@ -2497,7 +2558,8 @@
       <x:c r="C56" s="67"/>
       <x:c r="D56" s="44"/>
       <x:c r="E56" s="44"/>
-      <x:c r="F56" s="68"/>
+      <x:c r="F56" s="67"/>
+      <x:c r="G56" s="68"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="66"/>
@@ -2505,7 +2567,8 @@
       <x:c r="C57" s="67"/>
       <x:c r="D57" s="44"/>
       <x:c r="E57" s="44"/>
-      <x:c r="F57" s="68"/>
+      <x:c r="F57" s="67"/>
+      <x:c r="G57" s="68"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="66"/>
@@ -2513,7 +2576,8 @@
       <x:c r="C58" s="67"/>
       <x:c r="D58" s="44"/>
       <x:c r="E58" s="44"/>
-      <x:c r="F58" s="68"/>
+      <x:c r="F58" s="67"/>
+      <x:c r="G58" s="68"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="66"/>
@@ -2521,7 +2585,8 @@
       <x:c r="C59" s="67"/>
       <x:c r="D59" s="44"/>
       <x:c r="E59" s="44"/>
-      <x:c r="F59" s="68"/>
+      <x:c r="F59" s="67"/>
+      <x:c r="G59" s="68"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="66"/>
@@ -2529,7 +2594,8 @@
       <x:c r="C60" s="67"/>
       <x:c r="D60" s="44"/>
       <x:c r="E60" s="44"/>
-      <x:c r="F60" s="68"/>
+      <x:c r="F60" s="67"/>
+      <x:c r="G60" s="68"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="66"/>
@@ -2537,7 +2603,8 @@
       <x:c r="C61" s="67"/>
       <x:c r="D61" s="44"/>
       <x:c r="E61" s="44"/>
-      <x:c r="F61" s="68"/>
+      <x:c r="F61" s="67"/>
+      <x:c r="G61" s="68"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="66"/>
@@ -2545,7 +2612,8 @@
       <x:c r="C62" s="67"/>
       <x:c r="D62" s="44"/>
       <x:c r="E62" s="44"/>
-      <x:c r="F62" s="68"/>
+      <x:c r="F62" s="67"/>
+      <x:c r="G62" s="68"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="66"/>
@@ -2553,7 +2621,8 @@
       <x:c r="C63" s="67"/>
       <x:c r="D63" s="44"/>
       <x:c r="E63" s="44"/>
-      <x:c r="F63" s="68"/>
+      <x:c r="F63" s="67"/>
+      <x:c r="G63" s="68"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="66"/>
@@ -2561,7 +2630,8 @@
       <x:c r="C64" s="67"/>
       <x:c r="D64" s="44"/>
       <x:c r="E64" s="44"/>
-      <x:c r="F64" s="68"/>
+      <x:c r="F64" s="67"/>
+      <x:c r="G64" s="68"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="66"/>
@@ -2569,7 +2639,8 @@
       <x:c r="C65" s="67"/>
       <x:c r="D65" s="44"/>
       <x:c r="E65" s="44"/>
-      <x:c r="F65" s="68"/>
+      <x:c r="F65" s="67"/>
+      <x:c r="G65" s="68"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="66"/>
@@ -2577,7 +2648,8 @@
       <x:c r="C66" s="67"/>
       <x:c r="D66" s="44"/>
       <x:c r="E66" s="44"/>
-      <x:c r="F66" s="68"/>
+      <x:c r="F66" s="67"/>
+      <x:c r="G66" s="68"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="66"/>
@@ -2585,7 +2657,8 @@
       <x:c r="C67" s="67"/>
       <x:c r="D67" s="44"/>
       <x:c r="E67" s="44"/>
-      <x:c r="F67" s="68"/>
+      <x:c r="F67" s="67"/>
+      <x:c r="G67" s="68"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="66"/>
@@ -2593,7 +2666,8 @@
       <x:c r="C68" s="67"/>
       <x:c r="D68" s="44"/>
       <x:c r="E68" s="44"/>
-      <x:c r="F68" s="68"/>
+      <x:c r="F68" s="67"/>
+      <x:c r="G68" s="68"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="66"/>
@@ -2601,7 +2675,8 @@
       <x:c r="C69" s="67"/>
       <x:c r="D69" s="44"/>
       <x:c r="E69" s="44"/>
-      <x:c r="F69" s="68"/>
+      <x:c r="F69" s="67"/>
+      <x:c r="G69" s="68"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="66"/>
@@ -2609,7 +2684,8 @@
       <x:c r="C70" s="67"/>
       <x:c r="D70" s="44"/>
       <x:c r="E70" s="44"/>
-      <x:c r="F70" s="68"/>
+      <x:c r="F70" s="67"/>
+      <x:c r="G70" s="68"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="66"/>
@@ -2617,7 +2693,8 @@
       <x:c r="C71" s="67"/>
       <x:c r="D71" s="44"/>
       <x:c r="E71" s="44"/>
-      <x:c r="F71" s="68"/>
+      <x:c r="F71" s="67"/>
+      <x:c r="G71" s="68"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="66"/>
@@ -2625,7 +2702,8 @@
       <x:c r="C72" s="67"/>
       <x:c r="D72" s="44"/>
       <x:c r="E72" s="44"/>
-      <x:c r="F72" s="68"/>
+      <x:c r="F72" s="67"/>
+      <x:c r="G72" s="68"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="66"/>
@@ -2633,7 +2711,8 @@
       <x:c r="C73" s="67"/>
       <x:c r="D73" s="44"/>
       <x:c r="E73" s="44"/>
-      <x:c r="F73" s="68"/>
+      <x:c r="F73" s="67"/>
+      <x:c r="G73" s="68"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="66"/>
@@ -2641,7 +2720,8 @@
       <x:c r="C74" s="67"/>
       <x:c r="D74" s="44"/>
       <x:c r="E74" s="44"/>
-      <x:c r="F74" s="68"/>
+      <x:c r="F74" s="67"/>
+      <x:c r="G74" s="68"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="66"/>
@@ -2649,7 +2729,8 @@
       <x:c r="C75" s="67"/>
       <x:c r="D75" s="44"/>
       <x:c r="E75" s="44"/>
-      <x:c r="F75" s="68"/>
+      <x:c r="F75" s="67"/>
+      <x:c r="G75" s="68"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="66"/>
@@ -2657,7 +2738,8 @@
       <x:c r="C76" s="67"/>
       <x:c r="D76" s="44"/>
       <x:c r="E76" s="44"/>
-      <x:c r="F76" s="68"/>
+      <x:c r="F76" s="67"/>
+      <x:c r="G76" s="68"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="66"/>
@@ -2665,7 +2747,8 @@
       <x:c r="C77" s="67"/>
       <x:c r="D77" s="44"/>
       <x:c r="E77" s="44"/>
-      <x:c r="F77" s="68"/>
+      <x:c r="F77" s="67"/>
+      <x:c r="G77" s="68"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="66"/>
@@ -2673,7 +2756,8 @@
       <x:c r="C78" s="67"/>
       <x:c r="D78" s="44"/>
       <x:c r="E78" s="44"/>
-      <x:c r="F78" s="68"/>
+      <x:c r="F78" s="67"/>
+      <x:c r="G78" s="68"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="66"/>
@@ -2681,7 +2765,8 @@
       <x:c r="C79" s="67"/>
       <x:c r="D79" s="44"/>
       <x:c r="E79" s="44"/>
-      <x:c r="F79" s="68"/>
+      <x:c r="F79" s="67"/>
+      <x:c r="G79" s="68"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="66"/>
@@ -2689,7 +2774,8 @@
       <x:c r="C80" s="67"/>
       <x:c r="D80" s="44"/>
       <x:c r="E80" s="44"/>
-      <x:c r="F80" s="68"/>
+      <x:c r="F80" s="67"/>
+      <x:c r="G80" s="68"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="66"/>
@@ -2697,7 +2783,8 @@
       <x:c r="C81" s="67"/>
       <x:c r="D81" s="44"/>
       <x:c r="E81" s="44"/>
-      <x:c r="F81" s="68"/>
+      <x:c r="F81" s="67"/>
+      <x:c r="G81" s="68"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="66"/>
@@ -2705,7 +2792,8 @@
       <x:c r="C82" s="67"/>
       <x:c r="D82" s="44"/>
       <x:c r="E82" s="44"/>
-      <x:c r="F82" s="68"/>
+      <x:c r="F82" s="67"/>
+      <x:c r="G82" s="68"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="66"/>
@@ -2713,7 +2801,8 @@
       <x:c r="C83" s="67"/>
       <x:c r="D83" s="44"/>
       <x:c r="E83" s="44"/>
-      <x:c r="F83" s="68"/>
+      <x:c r="F83" s="67"/>
+      <x:c r="G83" s="68"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="66"/>
@@ -2721,7 +2810,8 @@
       <x:c r="C84" s="67"/>
       <x:c r="D84" s="44"/>
       <x:c r="E84" s="44"/>
-      <x:c r="F84" s="68"/>
+      <x:c r="F84" s="67"/>
+      <x:c r="G84" s="68"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="66"/>
@@ -2729,7 +2819,8 @@
       <x:c r="C85" s="67"/>
       <x:c r="D85" s="44"/>
       <x:c r="E85" s="44"/>
-      <x:c r="F85" s="68"/>
+      <x:c r="F85" s="67"/>
+      <x:c r="G85" s="68"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="66"/>
@@ -2737,7 +2828,8 @@
       <x:c r="C86" s="67"/>
       <x:c r="D86" s="44"/>
       <x:c r="E86" s="44"/>
-      <x:c r="F86" s="68"/>
+      <x:c r="F86" s="67"/>
+      <x:c r="G86" s="68"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="66"/>
@@ -2745,7 +2837,8 @@
       <x:c r="C87" s="67"/>
       <x:c r="D87" s="44"/>
       <x:c r="E87" s="44"/>
-      <x:c r="F87" s="68"/>
+      <x:c r="F87" s="67"/>
+      <x:c r="G87" s="68"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="66"/>
@@ -2753,7 +2846,8 @@
       <x:c r="C88" s="67"/>
       <x:c r="D88" s="44"/>
       <x:c r="E88" s="44"/>
-      <x:c r="F88" s="68"/>
+      <x:c r="F88" s="67"/>
+      <x:c r="G88" s="68"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="66"/>
@@ -2761,7 +2855,8 @@
       <x:c r="C89" s="67"/>
       <x:c r="D89" s="44"/>
       <x:c r="E89" s="44"/>
-      <x:c r="F89" s="68"/>
+      <x:c r="F89" s="67"/>
+      <x:c r="G89" s="68"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="66"/>
@@ -2769,7 +2864,8 @@
       <x:c r="C90" s="67"/>
       <x:c r="D90" s="44"/>
       <x:c r="E90" s="44"/>
-      <x:c r="F90" s="68"/>
+      <x:c r="F90" s="67"/>
+      <x:c r="G90" s="68"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="66"/>
@@ -2777,7 +2873,8 @@
       <x:c r="C91" s="67"/>
       <x:c r="D91" s="44"/>
       <x:c r="E91" s="44"/>
-      <x:c r="F91" s="68"/>
+      <x:c r="F91" s="67"/>
+      <x:c r="G91" s="68"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="66"/>
@@ -2785,7 +2882,8 @@
       <x:c r="C92" s="67"/>
       <x:c r="D92" s="44"/>
       <x:c r="E92" s="44"/>
-      <x:c r="F92" s="68"/>
+      <x:c r="F92" s="67"/>
+      <x:c r="G92" s="68"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="66"/>
@@ -2793,7 +2891,8 @@
       <x:c r="C93" s="67"/>
       <x:c r="D93" s="44"/>
       <x:c r="E93" s="44"/>
-      <x:c r="F93" s="68"/>
+      <x:c r="F93" s="67"/>
+      <x:c r="G93" s="68"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="66"/>
@@ -2801,7 +2900,8 @@
       <x:c r="C94" s="67"/>
       <x:c r="D94" s="44"/>
       <x:c r="E94" s="44"/>
-      <x:c r="F94" s="68"/>
+      <x:c r="F94" s="67"/>
+      <x:c r="G94" s="68"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="66"/>
@@ -2809,7 +2909,8 @@
       <x:c r="C95" s="67"/>
       <x:c r="D95" s="44"/>
       <x:c r="E95" s="44"/>
-      <x:c r="F95" s="68"/>
+      <x:c r="F95" s="67"/>
+      <x:c r="G95" s="68"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="66"/>
@@ -2817,7 +2918,8 @@
       <x:c r="C96" s="67"/>
       <x:c r="D96" s="44"/>
       <x:c r="E96" s="44"/>
-      <x:c r="F96" s="68"/>
+      <x:c r="F96" s="67"/>
+      <x:c r="G96" s="68"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="66"/>
@@ -2825,7 +2927,8 @@
       <x:c r="C97" s="67"/>
       <x:c r="D97" s="44"/>
       <x:c r="E97" s="44"/>
-      <x:c r="F97" s="68"/>
+      <x:c r="F97" s="67"/>
+      <x:c r="G97" s="68"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="66"/>
@@ -2833,7 +2936,8 @@
       <x:c r="C98" s="67"/>
       <x:c r="D98" s="44"/>
       <x:c r="E98" s="44"/>
-      <x:c r="F98" s="68"/>
+      <x:c r="F98" s="67"/>
+      <x:c r="G98" s="68"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="66"/>
@@ -2841,7 +2945,8 @@
       <x:c r="C99" s="67"/>
       <x:c r="D99" s="44"/>
       <x:c r="E99" s="44"/>
-      <x:c r="F99" s="68"/>
+      <x:c r="F99" s="67"/>
+      <x:c r="G99" s="68"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="77"/>
@@ -2849,21 +2954,22 @@
       <x:c r="C100" s="78"/>
       <x:c r="D100" s="79"/>
       <x:c r="E100" s="79"/>
-      <x:c r="F100" s="80"/>
+      <x:c r="F100" s="78"/>
+      <x:c r="G100" s="80"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:F1"/>
-    <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
   </x:mergeCells>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="F5:F100">
+    <x:dataValidation type="list" sqref="G5:G100">
       <x:formula1>"1,0"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2a6d9c46afd46ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03c22366b129498a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3630,7 +3736,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e9539354e174fdc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62e91a9a3bdd4d69"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>